<commit_message>
Actualización agosto indicadores médicos
</commit_message>
<xml_diff>
--- a/Dashboard.xlsx
+++ b/Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio\Desktop\NUEVO\DashboardMedico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0ED85C7-1BD5-404E-9B3B-6155BA643C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8325A96-8272-41E3-A8F6-CCEFFB9E8D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1407A859-4935-4127-A91B-F2429559B5A8}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="51">
   <si>
     <t>mes</t>
   </si>
@@ -194,6 +194,9 @@
   <si>
     <t>julio</t>
   </si>
+  <si>
+    <t>agosto</t>
+  </si>
 </sst>
 </file>
 
@@ -244,7 +247,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -323,8 +326,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="34">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -753,12 +762,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -967,22 +1002,31 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -991,10 +1035,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1009,26 +1053,24 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1037,13 +1079,13 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -10335,7 +10377,352 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+  <location ref="G26:I31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Suma de % De remisiones" fld="20" baseField="0" baseItem="0"/>
+    <dataField name="Suma de Total  de resolutividad" fld="21" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="3">
+    <format dxfId="2">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea field="0" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisRow" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="8" format="14" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="15" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10488,8 +10875,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E3:L8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10597,7 +10984,7 @@
     <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="1">
+    <format dxfId="4">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -10607,7 +10994,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="3">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -10623,351 +11010,6 @@
       </pivotArea>
     </format>
   </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="G26:I31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Suma de % De remisiones" fld="20" baseField="0" baseItem="0"/>
-    <dataField name="Suma de Total  de resolutividad" fld="21" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="3">
-    <format dxfId="4">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="3">
-      <pivotArea field="0" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisRow" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="2">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="8" format="14" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="8" format="15" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -11342,7 +11384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FD4F9-2910-4648-84AF-C941CDDEB3D5}">
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:V70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="11.42578125" style="60"/>
@@ -11383,10 +11425,10 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="90" t="s">
+      <c r="K1" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="91"/>
+      <c r="L1" s="82"/>
       <c r="M1" s="63" t="s">
         <v>11</v>
       </c>
@@ -11515,7 +11557,7 @@
         <v>2</v>
       </c>
       <c r="G3" s="64">
-        <f t="shared" ref="G3:G61" si="1">E3/D3</f>
+        <f t="shared" ref="G3:G66" si="1">E3/D3</f>
         <v>0.8</v>
       </c>
       <c r="H3" s="14">
@@ -11529,44 +11571,44 @@
       <c r="J3" s="16">
         <v>60</v>
       </c>
-      <c r="K3" s="84">
+      <c r="K3" s="83">
         <v>8</v>
       </c>
-      <c r="L3" s="85"/>
+      <c r="L3" s="84"/>
       <c r="M3" s="64">
-        <f t="shared" ref="M3:M61" si="3">J3/I3</f>
+        <f t="shared" ref="M3:M66" si="3">J3/I3</f>
         <v>0.88235294117647056</v>
       </c>
       <c r="N3" s="17">
         <v>55</v>
       </c>
       <c r="O3" s="66">
-        <f t="shared" ref="O3:O61" si="4">N3/J3</f>
+        <f t="shared" ref="O3:O66" si="4">N3/J3</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="P3" s="16">
         <v>4</v>
       </c>
       <c r="Q3" s="66">
-        <f t="shared" ref="Q3:Q61" si="5">P3/J3</f>
+        <f t="shared" ref="Q3:Q66" si="5">P3/J3</f>
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="R3" s="16">
         <v>2</v>
       </c>
       <c r="S3" s="67">
-        <f t="shared" ref="S3:S61" si="6">R3/J3</f>
+        <f t="shared" ref="S3:S66" si="6">R3/J3</f>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="T3" s="14">
         <v>7</v>
       </c>
       <c r="U3" s="66">
-        <f t="shared" ref="U3:U61" si="7">T3/J3</f>
+        <f t="shared" ref="U3:U66" si="7">T3/J3</f>
         <v>0.11666666666666667</v>
       </c>
       <c r="V3" s="68">
-        <f t="shared" ref="V3:V61" si="8">(1-(T3/J3))</f>
+        <f t="shared" ref="V3:V66" si="8">(1-(T3/J3))</f>
         <v>0.8833333333333333</v>
       </c>
     </row>
@@ -11605,10 +11647,10 @@
       <c r="J4" s="11">
         <v>50</v>
       </c>
-      <c r="K4" s="80">
+      <c r="K4" s="79">
         <v>10</v>
       </c>
-      <c r="L4" s="81"/>
+      <c r="L4" s="80"/>
       <c r="M4" s="64">
         <f t="shared" si="3"/>
         <v>0.83333333333333337</v>
@@ -11681,10 +11723,10 @@
       <c r="J5" s="11">
         <v>18</v>
       </c>
-      <c r="K5" s="80">
+      <c r="K5" s="79">
         <v>3</v>
       </c>
-      <c r="L5" s="81"/>
+      <c r="L5" s="80"/>
       <c r="M5" s="64">
         <f t="shared" si="3"/>
         <v>0.8571428571428571</v>
@@ -11757,10 +11799,10 @@
       <c r="J6" s="20">
         <v>44</v>
       </c>
-      <c r="K6" s="82">
+      <c r="K6" s="85">
         <v>11</v>
       </c>
-      <c r="L6" s="83"/>
+      <c r="L6" s="86"/>
       <c r="M6" s="64">
         <f t="shared" si="3"/>
         <v>0.8</v>
@@ -11833,10 +11875,10 @@
       <c r="J7" s="16">
         <v>10</v>
       </c>
-      <c r="K7" s="84">
+      <c r="K7" s="83">
         <v>1</v>
       </c>
-      <c r="L7" s="85"/>
+      <c r="L7" s="84"/>
       <c r="M7" s="64">
         <f t="shared" si="3"/>
         <v>0.90909090909090906</v>
@@ -11909,10 +11951,10 @@
       <c r="J8" s="27">
         <v>8</v>
       </c>
-      <c r="K8" s="92">
+      <c r="K8" s="87">
         <v>1</v>
       </c>
-      <c r="L8" s="93"/>
+      <c r="L8" s="88"/>
       <c r="M8" s="64">
         <f t="shared" si="3"/>
         <v>0.88888888888888884</v>
@@ -12061,10 +12103,10 @@
       <c r="J10" s="16">
         <v>112</v>
       </c>
-      <c r="K10" s="84">
+      <c r="K10" s="83">
         <v>2</v>
       </c>
-      <c r="L10" s="85"/>
+      <c r="L10" s="84"/>
       <c r="M10" s="64">
         <f t="shared" si="3"/>
         <v>0.98245614035087714</v>
@@ -12137,10 +12179,10 @@
       <c r="J11" s="11">
         <v>77</v>
       </c>
-      <c r="K11" s="80">
+      <c r="K11" s="79">
         <v>1</v>
       </c>
-      <c r="L11" s="81"/>
+      <c r="L11" s="80"/>
       <c r="M11" s="64">
         <f t="shared" si="3"/>
         <v>0.98717948717948723</v>
@@ -12213,10 +12255,10 @@
       <c r="J12" s="11">
         <v>61</v>
       </c>
-      <c r="K12" s="80">
+      <c r="K12" s="79">
         <v>4</v>
       </c>
-      <c r="L12" s="81"/>
+      <c r="L12" s="80"/>
       <c r="M12" s="64">
         <f t="shared" si="3"/>
         <v>0.93846153846153846</v>
@@ -12289,10 +12331,10 @@
       <c r="J13" s="20">
         <v>64</v>
       </c>
-      <c r="K13" s="82">
+      <c r="K13" s="85">
         <v>1</v>
       </c>
-      <c r="L13" s="83"/>
+      <c r="L13" s="86"/>
       <c r="M13" s="64">
         <f t="shared" si="3"/>
         <v>0.98461538461538467</v>
@@ -12365,10 +12407,10 @@
       <c r="J14" s="16">
         <v>21</v>
       </c>
-      <c r="K14" s="84">
+      <c r="K14" s="83">
         <v>1</v>
       </c>
-      <c r="L14" s="85"/>
+      <c r="L14" s="84"/>
       <c r="M14" s="64">
         <f t="shared" si="3"/>
         <v>0.95454545454545459</v>
@@ -12440,10 +12482,10 @@
       <c r="J15" s="34">
         <v>28</v>
       </c>
-      <c r="K15" s="86">
+      <c r="K15" s="89">
         <v>0</v>
       </c>
-      <c r="L15" s="87"/>
+      <c r="L15" s="90"/>
       <c r="M15" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -12516,10 +12558,10 @@
       <c r="J16" s="40">
         <v>23</v>
       </c>
-      <c r="K16" s="88">
+      <c r="K16" s="91">
         <v>1</v>
       </c>
-      <c r="L16" s="89"/>
+      <c r="L16" s="92"/>
       <c r="M16" s="64">
         <f t="shared" si="3"/>
         <v>0.95833333333333337</v>
@@ -12668,10 +12710,10 @@
       <c r="J18" s="16">
         <v>133</v>
       </c>
-      <c r="K18" s="84">
+      <c r="K18" s="83">
         <v>2</v>
       </c>
-      <c r="L18" s="85"/>
+      <c r="L18" s="84"/>
       <c r="M18" s="64">
         <f t="shared" si="3"/>
         <v>0.98518518518518516</v>
@@ -12744,10 +12786,10 @@
       <c r="J19" s="11">
         <v>111</v>
       </c>
-      <c r="K19" s="80">
+      <c r="K19" s="79">
         <v>1</v>
       </c>
-      <c r="L19" s="81"/>
+      <c r="L19" s="80"/>
       <c r="M19" s="64">
         <f t="shared" si="3"/>
         <v>0.9910714285714286</v>
@@ -12820,10 +12862,10 @@
       <c r="J20" s="11">
         <v>76</v>
       </c>
-      <c r="K20" s="80">
+      <c r="K20" s="79">
         <v>1</v>
       </c>
-      <c r="L20" s="81"/>
+      <c r="L20" s="80"/>
       <c r="M20" s="64">
         <f t="shared" si="3"/>
         <v>0.98701298701298701</v>
@@ -12895,10 +12937,10 @@
       <c r="J21" s="11">
         <v>43</v>
       </c>
-      <c r="K21" s="80">
+      <c r="K21" s="79">
         <v>2</v>
       </c>
-      <c r="L21" s="81"/>
+      <c r="L21" s="80"/>
       <c r="M21" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -12971,10 +13013,10 @@
       <c r="J22" s="20">
         <v>86</v>
       </c>
-      <c r="K22" s="82">
+      <c r="K22" s="85">
         <v>1</v>
       </c>
-      <c r="L22" s="83"/>
+      <c r="L22" s="86"/>
       <c r="M22" s="64">
         <f t="shared" si="3"/>
         <v>0.9885057471264368</v>
@@ -13047,10 +13089,10 @@
       <c r="J23" s="16">
         <v>26</v>
       </c>
-      <c r="K23" s="84">
+      <c r="K23" s="83">
         <v>1</v>
       </c>
-      <c r="L23" s="85"/>
+      <c r="L23" s="84"/>
       <c r="M23" s="64">
         <f t="shared" si="3"/>
         <v>0.96296296296296291</v>
@@ -13122,10 +13164,10 @@
       <c r="J24" s="34">
         <v>30</v>
       </c>
-      <c r="K24" s="86">
+      <c r="K24" s="89">
         <v>0</v>
       </c>
-      <c r="L24" s="87"/>
+      <c r="L24" s="90"/>
       <c r="M24" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13198,10 +13240,10 @@
       <c r="J25" s="49">
         <v>43</v>
       </c>
-      <c r="K25" s="76">
+      <c r="K25" s="93">
         <v>2</v>
       </c>
-      <c r="L25" s="77"/>
+      <c r="L25" s="94"/>
       <c r="M25" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -13273,11 +13315,11 @@
       <c r="J26" s="56">
         <v>143</v>
       </c>
-      <c r="K26" s="78">
+      <c r="K26" s="95">
         <f>I26-J26</f>
         <v>6</v>
       </c>
-      <c r="L26" s="79"/>
+      <c r="L26" s="96"/>
       <c r="M26" s="64">
         <f t="shared" si="3"/>
         <v>0.95973154362416102</v>
@@ -13955,10 +13997,10 @@
       <c r="J35">
         <v>134</v>
       </c>
-      <c r="K35" s="94">
+      <c r="K35" s="76">
         <v>27</v>
       </c>
-      <c r="L35" s="94"/>
+      <c r="L35" s="76"/>
       <c r="M35" s="64">
         <f t="shared" si="3"/>
         <v>0.83229813664596275</v>
@@ -14028,10 +14070,10 @@
       <c r="J36">
         <v>118</v>
       </c>
-      <c r="K36" s="95">
+      <c r="K36" s="77">
         <v>33</v>
       </c>
-      <c r="L36" s="95"/>
+      <c r="L36" s="77"/>
       <c r="M36" s="64">
         <f t="shared" si="3"/>
         <v>0.7814569536423841</v>
@@ -14101,10 +14143,10 @@
       <c r="J37">
         <v>86</v>
       </c>
-      <c r="K37" s="95">
+      <c r="K37" s="77">
         <v>40</v>
       </c>
-      <c r="L37" s="95"/>
+      <c r="L37" s="77"/>
       <c r="M37" s="64">
         <f t="shared" si="3"/>
         <v>0.68253968253968256</v>
@@ -14174,10 +14216,10 @@
       <c r="J38">
         <v>91</v>
       </c>
-      <c r="K38" s="95">
+      <c r="K38" s="77">
         <v>35</v>
       </c>
-      <c r="L38" s="95"/>
+      <c r="L38" s="77"/>
       <c r="M38" s="64">
         <f t="shared" si="3"/>
         <v>0.72222222222222221</v>
@@ -14247,10 +14289,10 @@
       <c r="J39">
         <v>92</v>
       </c>
-      <c r="K39" s="95">
+      <c r="K39" s="77">
         <v>38</v>
       </c>
-      <c r="L39" s="95"/>
+      <c r="L39" s="77"/>
       <c r="M39" s="64">
         <f t="shared" si="3"/>
         <v>0.70769230769230773</v>
@@ -14320,10 +14362,10 @@
       <c r="J40">
         <v>53</v>
       </c>
-      <c r="K40" s="95">
+      <c r="K40" s="77">
         <v>23</v>
       </c>
-      <c r="L40" s="95"/>
+      <c r="L40" s="77"/>
       <c r="M40" s="64">
         <f t="shared" si="3"/>
         <v>0.69736842105263153</v>
@@ -14393,10 +14435,10 @@
       <c r="J41">
         <v>29</v>
       </c>
-      <c r="K41" s="95">
+      <c r="K41" s="77">
         <v>5</v>
       </c>
-      <c r="L41" s="95"/>
+      <c r="L41" s="77"/>
       <c r="M41" s="64">
         <f t="shared" si="3"/>
         <v>0.8529411764705882</v>
@@ -14466,10 +14508,10 @@
       <c r="J42">
         <v>22</v>
       </c>
-      <c r="K42" s="95">
+      <c r="K42" s="77">
         <v>7</v>
       </c>
-      <c r="L42" s="95"/>
+      <c r="L42" s="77"/>
       <c r="M42" s="64">
         <f t="shared" si="3"/>
         <v>0.75862068965517238</v>
@@ -14539,10 +14581,10 @@
       <c r="J43">
         <v>40</v>
       </c>
-      <c r="K43" s="96">
+      <c r="K43" s="78">
         <v>20</v>
       </c>
-      <c r="L43" s="96"/>
+      <c r="L43" s="78"/>
       <c r="M43" s="64">
         <f t="shared" si="3"/>
         <v>0.66666666666666663</v>
@@ -15948,17 +15990,737 @@
         <v>0.95</v>
       </c>
     </row>
+    <row r="62" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B62" t="s">
+        <v>22</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D62" s="9">
+        <v>19</v>
+      </c>
+      <c r="E62" s="10">
+        <v>18</v>
+      </c>
+      <c r="F62" s="11">
+        <f>D62-E62</f>
+        <v>1</v>
+      </c>
+      <c r="G62" s="64">
+        <f t="shared" si="1"/>
+        <v>0.94736842105263153</v>
+      </c>
+      <c r="H62" s="9">
+        <f>E62*4*3</f>
+        <v>216</v>
+      </c>
+      <c r="I62" s="11">
+        <f>J62+K62</f>
+        <v>167</v>
+      </c>
+      <c r="J62" s="70">
+        <v>130</v>
+      </c>
+      <c r="K62" s="74">
+        <v>37</v>
+      </c>
+      <c r="L62" s="75"/>
+      <c r="M62" s="64">
+        <f t="shared" si="3"/>
+        <v>0.77844311377245512</v>
+      </c>
+      <c r="N62" s="12">
+        <v>75</v>
+      </c>
+      <c r="O62" s="66">
+        <f t="shared" si="4"/>
+        <v>0.57692307692307687</v>
+      </c>
+      <c r="P62" s="11">
+        <v>33</v>
+      </c>
+      <c r="Q62" s="66">
+        <f t="shared" si="5"/>
+        <v>0.25384615384615383</v>
+      </c>
+      <c r="R62" s="11">
+        <v>9</v>
+      </c>
+      <c r="S62" s="67">
+        <f t="shared" si="6"/>
+        <v>6.9230769230769235E-2</v>
+      </c>
+      <c r="T62" s="9">
+        <v>16</v>
+      </c>
+      <c r="U62" s="66">
+        <f t="shared" si="7"/>
+        <v>0.12307692307692308</v>
+      </c>
+      <c r="V62" s="68">
+        <f t="shared" si="8"/>
+        <v>0.87692307692307692</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B63" t="s">
+        <v>22</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D63" s="14">
+        <v>19</v>
+      </c>
+      <c r="E63" s="15">
+        <v>17</v>
+      </c>
+      <c r="F63" s="11">
+        <f t="shared" ref="F63:F65" si="29">D63-E63</f>
+        <v>2</v>
+      </c>
+      <c r="G63" s="64">
+        <f t="shared" si="1"/>
+        <v>0.89473684210526316</v>
+      </c>
+      <c r="H63" s="14">
+        <f>E63*4*2</f>
+        <v>136</v>
+      </c>
+      <c r="I63" s="11">
+        <f>J63+K63</f>
+        <v>142</v>
+      </c>
+      <c r="J63" s="70">
+        <v>105</v>
+      </c>
+      <c r="K63" s="74">
+        <v>37</v>
+      </c>
+      <c r="L63" s="75"/>
+      <c r="M63" s="64">
+        <f t="shared" si="3"/>
+        <v>0.73943661971830987</v>
+      </c>
+      <c r="N63" s="17">
+        <v>115</v>
+      </c>
+      <c r="O63" s="66">
+        <f t="shared" si="4"/>
+        <v>1.0952380952380953</v>
+      </c>
+      <c r="P63" s="16">
+        <v>182</v>
+      </c>
+      <c r="Q63" s="66">
+        <f t="shared" si="5"/>
+        <v>1.7333333333333334</v>
+      </c>
+      <c r="R63" s="16">
+        <v>6</v>
+      </c>
+      <c r="S63" s="67">
+        <f t="shared" si="6"/>
+        <v>5.7142857142857141E-2</v>
+      </c>
+      <c r="T63" s="14">
+        <v>18</v>
+      </c>
+      <c r="U63" s="66">
+        <f t="shared" si="7"/>
+        <v>0.17142857142857143</v>
+      </c>
+      <c r="V63" s="68">
+        <f t="shared" si="8"/>
+        <v>0.82857142857142851</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B64" t="s">
+        <v>22</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D64" s="9">
+        <v>19</v>
+      </c>
+      <c r="E64" s="10">
+        <v>17</v>
+      </c>
+      <c r="F64" s="11">
+        <f t="shared" si="29"/>
+        <v>2</v>
+      </c>
+      <c r="G64" s="64">
+        <f t="shared" si="1"/>
+        <v>0.89473684210526316</v>
+      </c>
+      <c r="H64" s="9">
+        <f>E64*4*2</f>
+        <v>136</v>
+      </c>
+      <c r="I64" s="11">
+        <f>J64+K64</f>
+        <v>117</v>
+      </c>
+      <c r="J64" s="70">
+        <v>78</v>
+      </c>
+      <c r="K64" s="74">
+        <v>39</v>
+      </c>
+      <c r="L64" s="75"/>
+      <c r="M64" s="64">
+        <f t="shared" si="3"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="N64" s="12">
+        <v>118</v>
+      </c>
+      <c r="O64" s="66">
+        <f t="shared" si="4"/>
+        <v>1.5128205128205128</v>
+      </c>
+      <c r="P64" s="11">
+        <v>12</v>
+      </c>
+      <c r="Q64" s="66">
+        <f t="shared" si="5"/>
+        <v>0.15384615384615385</v>
+      </c>
+      <c r="R64" s="11">
+        <v>4</v>
+      </c>
+      <c r="S64" s="67">
+        <f t="shared" si="6"/>
+        <v>5.128205128205128E-2</v>
+      </c>
+      <c r="T64" s="9">
+        <v>6</v>
+      </c>
+      <c r="U64" s="66">
+        <f t="shared" si="7"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="V64" s="68">
+        <f t="shared" si="8"/>
+        <v>0.92307692307692313</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B65" t="s">
+        <v>22</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D65" s="9">
+        <v>19</v>
+      </c>
+      <c r="E65" s="10">
+        <v>18</v>
+      </c>
+      <c r="F65" s="11">
+        <f t="shared" si="29"/>
+        <v>1</v>
+      </c>
+      <c r="G65" s="64">
+        <f t="shared" si="1"/>
+        <v>0.94736842105263153</v>
+      </c>
+      <c r="H65" s="9">
+        <f>E65*4*2</f>
+        <v>144</v>
+      </c>
+      <c r="I65" s="11">
+        <f t="shared" ref="I65:I70" si="30">J65+K65</f>
+        <v>104</v>
+      </c>
+      <c r="J65" s="70">
+        <v>73</v>
+      </c>
+      <c r="K65" s="74">
+        <v>31</v>
+      </c>
+      <c r="L65" s="75"/>
+      <c r="M65" s="64">
+        <f t="shared" si="3"/>
+        <v>0.70192307692307687</v>
+      </c>
+      <c r="N65" s="12">
+        <v>91</v>
+      </c>
+      <c r="O65" s="66">
+        <f t="shared" si="4"/>
+        <v>1.2465753424657535</v>
+      </c>
+      <c r="P65" s="11">
+        <v>60</v>
+      </c>
+      <c r="Q65" s="66">
+        <f t="shared" si="5"/>
+        <v>0.82191780821917804</v>
+      </c>
+      <c r="R65" s="11">
+        <v>3</v>
+      </c>
+      <c r="S65" s="67">
+        <f t="shared" si="6"/>
+        <v>4.1095890410958902E-2</v>
+      </c>
+      <c r="T65" s="9">
+        <v>5</v>
+      </c>
+      <c r="U65" s="66">
+        <f t="shared" si="7"/>
+        <v>6.8493150684931503E-2</v>
+      </c>
+      <c r="V65" s="68">
+        <f t="shared" si="8"/>
+        <v>0.93150684931506844</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B66" t="s">
+        <v>35</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D66" s="9">
+        <v>19</v>
+      </c>
+      <c r="E66" s="10">
+        <v>17</v>
+      </c>
+      <c r="F66" s="11">
+        <f>D66-E66</f>
+        <v>2</v>
+      </c>
+      <c r="G66" s="64">
+        <f t="shared" si="1"/>
+        <v>0.89473684210526316</v>
+      </c>
+      <c r="H66" s="9">
+        <f>E66*3*2</f>
+        <v>102</v>
+      </c>
+      <c r="I66" s="11">
+        <f t="shared" si="30"/>
+        <v>157</v>
+      </c>
+      <c r="J66" s="70">
+        <v>119</v>
+      </c>
+      <c r="K66" s="74">
+        <v>38</v>
+      </c>
+      <c r="L66" s="75"/>
+      <c r="M66" s="64">
+        <f t="shared" si="3"/>
+        <v>0.7579617834394905</v>
+      </c>
+      <c r="N66" s="12">
+        <v>113</v>
+      </c>
+      <c r="O66" s="66">
+        <f t="shared" si="4"/>
+        <v>0.94957983193277307</v>
+      </c>
+      <c r="P66" s="11">
+        <v>160</v>
+      </c>
+      <c r="Q66" s="66">
+        <f t="shared" si="5"/>
+        <v>1.3445378151260505</v>
+      </c>
+      <c r="R66" s="11">
+        <v>29</v>
+      </c>
+      <c r="S66" s="67">
+        <f t="shared" si="6"/>
+        <v>0.24369747899159663</v>
+      </c>
+      <c r="T66" s="9">
+        <v>17</v>
+      </c>
+      <c r="U66" s="66">
+        <f t="shared" si="7"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="V66" s="68">
+        <f t="shared" si="8"/>
+        <v>0.85714285714285721</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B67" t="s">
+        <v>27</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D67" s="18">
+        <v>19</v>
+      </c>
+      <c r="E67" s="19">
+        <v>19</v>
+      </c>
+      <c r="F67" s="20">
+        <f>D67-E67</f>
+        <v>0</v>
+      </c>
+      <c r="G67" s="64">
+        <f t="shared" ref="G67:G70" si="31">E67/D67</f>
+        <v>1</v>
+      </c>
+      <c r="H67" s="18">
+        <f>E67*8*2</f>
+        <v>304</v>
+      </c>
+      <c r="I67" s="11">
+        <f t="shared" si="30"/>
+        <v>104</v>
+      </c>
+      <c r="J67" s="71">
+        <v>77</v>
+      </c>
+      <c r="K67" s="74">
+        <v>27</v>
+      </c>
+      <c r="L67" s="75"/>
+      <c r="M67" s="64">
+        <f t="shared" ref="M67:M70" si="32">J67/I67</f>
+        <v>0.74038461538461542</v>
+      </c>
+      <c r="N67" s="21">
+        <v>1</v>
+      </c>
+      <c r="O67" s="66">
+        <f t="shared" ref="O67:O70" si="33">N67/J67</f>
+        <v>1.2987012987012988E-2</v>
+      </c>
+      <c r="P67" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="66">
+        <f t="shared" ref="Q67:Q70" si="34">P67/J67</f>
+        <v>0</v>
+      </c>
+      <c r="R67" s="20">
+        <v>0</v>
+      </c>
+      <c r="S67" s="67">
+        <f t="shared" ref="S67:S70" si="35">R67/J67</f>
+        <v>0</v>
+      </c>
+      <c r="T67" s="18">
+        <v>12</v>
+      </c>
+      <c r="U67" s="66">
+        <f t="shared" ref="U67:U70" si="36">T67/J67</f>
+        <v>0.15584415584415584</v>
+      </c>
+      <c r="V67" s="68">
+        <f t="shared" ref="V67:V70" si="37">(1-(T67/J67))</f>
+        <v>0.8441558441558441</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B68" t="s">
+        <v>27</v>
+      </c>
+      <c r="C68" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D68" s="14">
+        <v>19</v>
+      </c>
+      <c r="E68" s="15">
+        <v>18</v>
+      </c>
+      <c r="F68" s="20">
+        <f t="shared" ref="F68:F69" si="38">D68-E68</f>
+        <v>1</v>
+      </c>
+      <c r="G68" s="64">
+        <f t="shared" si="31"/>
+        <v>0.94736842105263153</v>
+      </c>
+      <c r="H68" s="14">
+        <f>E68*4*2</f>
+        <v>144</v>
+      </c>
+      <c r="I68" s="11">
+        <f t="shared" si="30"/>
+        <v>64</v>
+      </c>
+      <c r="J68" s="70">
+        <v>44</v>
+      </c>
+      <c r="K68" s="98">
+        <v>20</v>
+      </c>
+      <c r="L68" s="99"/>
+      <c r="M68" s="64">
+        <f t="shared" si="32"/>
+        <v>0.6875</v>
+      </c>
+      <c r="N68" s="17">
+        <v>1</v>
+      </c>
+      <c r="O68" s="66">
+        <f t="shared" si="33"/>
+        <v>2.2727272727272728E-2</v>
+      </c>
+      <c r="P68" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="66">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="R68" s="16">
+        <v>0</v>
+      </c>
+      <c r="S68" s="67">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="T68" s="14">
+        <v>4</v>
+      </c>
+      <c r="U68" s="66">
+        <f t="shared" si="36"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="V68" s="68">
+        <f t="shared" si="37"/>
+        <v>0.90909090909090906</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B69" t="s">
+        <v>27</v>
+      </c>
+      <c r="C69" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="D69" s="32">
+        <v>19</v>
+      </c>
+      <c r="E69" s="33">
+        <v>13</v>
+      </c>
+      <c r="F69" s="20">
+        <f t="shared" si="38"/>
+        <v>6</v>
+      </c>
+      <c r="G69" s="64">
+        <f t="shared" si="31"/>
+        <v>0.68421052631578949</v>
+      </c>
+      <c r="H69" s="32">
+        <f>E69*4*2</f>
+        <v>104</v>
+      </c>
+      <c r="I69" s="11">
+        <f t="shared" si="30"/>
+        <v>43</v>
+      </c>
+      <c r="J69" s="72">
+        <v>24</v>
+      </c>
+      <c r="K69" s="74">
+        <v>19</v>
+      </c>
+      <c r="L69" s="75"/>
+      <c r="M69" s="64">
+        <f t="shared" si="32"/>
+        <v>0.55813953488372092</v>
+      </c>
+      <c r="N69" s="35">
+        <v>3</v>
+      </c>
+      <c r="O69" s="66">
+        <f t="shared" si="33"/>
+        <v>0.125</v>
+      </c>
+      <c r="P69" s="34">
+        <v>0</v>
+      </c>
+      <c r="Q69" s="66">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="R69" s="34">
+        <v>0</v>
+      </c>
+      <c r="S69" s="67">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="T69" s="32">
+        <v>2</v>
+      </c>
+      <c r="U69" s="66">
+        <f t="shared" si="36"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="V69" s="68">
+        <f t="shared" si="37"/>
+        <v>0.91666666666666663</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="97" t="s">
+        <v>50</v>
+      </c>
+      <c r="B70" t="s">
+        <v>30</v>
+      </c>
+      <c r="C70" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D70" s="45">
+        <v>14</v>
+      </c>
+      <c r="E70" s="46">
+        <v>14</v>
+      </c>
+      <c r="F70" s="47">
+        <f>D70-E70</f>
+        <v>0</v>
+      </c>
+      <c r="G70" s="64">
+        <f t="shared" si="31"/>
+        <v>1</v>
+      </c>
+      <c r="H70" s="45">
+        <f>E70*4*2</f>
+        <v>112</v>
+      </c>
+      <c r="I70" s="11">
+        <f t="shared" si="30"/>
+        <v>79</v>
+      </c>
+      <c r="J70" s="73">
+        <v>46</v>
+      </c>
+      <c r="K70" s="74">
+        <v>33</v>
+      </c>
+      <c r="L70" s="75"/>
+      <c r="M70" s="64">
+        <f t="shared" si="32"/>
+        <v>0.58227848101265822</v>
+      </c>
+      <c r="N70" s="35">
+        <v>0</v>
+      </c>
+      <c r="O70" s="66">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="P70" s="34">
+        <v>0</v>
+      </c>
+      <c r="Q70" s="66">
+        <f t="shared" si="34"/>
+        <v>0</v>
+      </c>
+      <c r="R70" s="49">
+        <v>0</v>
+      </c>
+      <c r="S70" s="67">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="T70" s="51">
+        <v>1</v>
+      </c>
+      <c r="U70" s="66">
+        <f t="shared" si="36"/>
+        <v>2.1739130434782608E-2</v>
+      </c>
+      <c r="V70" s="68">
+        <f t="shared" si="37"/>
+        <v>0.97826086956521741</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="61">
-    <mergeCell ref="K58:L58"/>
-    <mergeCell ref="K59:L59"/>
-    <mergeCell ref="K60:L60"/>
-    <mergeCell ref="K61:L61"/>
-    <mergeCell ref="K53:L53"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="K55:L55"/>
-    <mergeCell ref="K56:L56"/>
-    <mergeCell ref="K57:L57"/>
+  <mergeCells count="70">
+    <mergeCell ref="K67:L67"/>
+    <mergeCell ref="K68:L68"/>
+    <mergeCell ref="K69:L69"/>
+    <mergeCell ref="K70:L70"/>
+    <mergeCell ref="K62:L62"/>
+    <mergeCell ref="K63:L63"/>
+    <mergeCell ref="K64:L64"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="K66:L66"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="K48:L48"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K13:L13"/>
     <mergeCell ref="K49:L49"/>
     <mergeCell ref="K50:L50"/>
     <mergeCell ref="K51:L51"/>
@@ -15975,42 +16737,15 @@
     <mergeCell ref="K44:L44"/>
     <mergeCell ref="K45:L45"/>
     <mergeCell ref="K46:L46"/>
-    <mergeCell ref="K47:L47"/>
-    <mergeCell ref="K48:L48"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K58:L58"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="K60:L60"/>
+    <mergeCell ref="K61:L61"/>
+    <mergeCell ref="K53:L53"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="K55:L55"/>
+    <mergeCell ref="K56:L56"/>
+    <mergeCell ref="K57:L57"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>